<commit_message>
DATA. Actualizo predicciones para USA
</commit_message>
<xml_diff>
--- a/data/usa/p6_deployment/data_preparation/df_emergency_fill.xlsx
+++ b/data/usa/p6_deployment/data_preparation/df_emergency_fill.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,54 +436,74 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>mean_last_match_mean_rat_player_start_home_against</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>mean_last_match_mean_rat_player_start_away_against</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_age_player_sub</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_hei_player_start</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_int_rep_player_start</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_pot_player_sub</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_hei_player_sub</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_age_player_start</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_pot_player_start</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_rat_player_sub</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_int_rep_player_sub</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>dif_mean_val_player_sub</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>dif_mean_rat_player_start</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_pot_player_start</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_pot_player_sub</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_int_rep_player_start</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_age_player_start</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_val_player_sub</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_rat_player_sub</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>dif_mean_val_player_start</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>foKU4Bi8</t>
+          <t>YJuQfCBA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -496,11 +516,15 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>l8RwqFCb</t>
+          <t>GroLehd4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -513,11 +537,15 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>AHSZqech</t>
+          <t>xhnHdYtb</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -530,11 +558,15 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>xUcLQXdU</t>
+          <t>rVnDcERi</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -547,11 +579,15 @@
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>EkZQoHSu</t>
+          <t>URr9bfCo</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -564,11 +600,15 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>htYUpyrn</t>
+          <t>0n3Ddmal</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -581,11 +621,15 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>dKkDSgSH</t>
+          <t>SM4QZAZp</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -598,11 +642,15 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>A3m1Vera</t>
+          <t>QDIbviRT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -615,11 +663,15 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>8lOY3V6E</t>
+          <t>ImJfuXBN</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,11 +684,15 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>ITj9TZCB</t>
+          <t>dYUosgsB</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -649,11 +705,15 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>lfn5UFc5</t>
+          <t>U3Cs29yR</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -666,11 +726,15 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>vquIRDsO</t>
+          <t>vcKjtDdH</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -683,11 +747,15 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>jDDw3kMK</t>
+          <t>Me49cTqr</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -700,11 +768,15 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>trWntSE7</t>
+          <t>rVQsrZR4</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -717,11 +789,15 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>AoWGqXpJ</t>
+          <t>l8RwqFCb</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -734,11 +810,15 @@
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>SvbdWyTh</t>
+          <t>foKU4Bi8</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -751,11 +831,15 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>hIoLKAg0</t>
+          <t>AHSZqech</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -768,11 +852,15 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>KEflYcbt</t>
+          <t>xUcLQXdU</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -785,11 +873,15 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>EyfhXHDn</t>
+          <t>EkZQoHSu</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -802,6 +894,178 @@
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>htYUpyrn</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>vquIRDsO</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>lfn5UFc5</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>dKkDSgSH</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>ITj9TZCB</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>jDDw3kMK</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>8lOY3V6E</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>A3m1Vera</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>